<commit_message>
fix: incluir cuarto integrante en desplegables de responsable
</commit_message>
<xml_diff>
--- a/Contrato/AulaFlow_2_0_Contrato_operativo_v1.0.xlsx
+++ b/Contrato/AulaFlow_2_0_Contrato_operativo_v1.0.xlsx
@@ -2,25 +2,25 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Contrato" sheetId="1" r:id="R9c46432c4b284bef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 PI II" sheetId="2" r:id="R84544c0266414cd2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 AD" sheetId="3" r:id="R99ea35fa3c5445c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 PMDM" sheetId="4" r:id="R82c5e4165c374eb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Hitos" sheetId="5" r:id="R2013a2041b50420c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99 Guía" sheetId="6" r:id="Rf2b60ee82511447c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 DI" sheetId="7" r:id="Rd2bbc16e54d14b2b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 PSP" sheetId="8" r:id="R2eddb53b49844b9a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 SGE" sheetId="9" r:id="R1c95e94370e341ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Nube" sheetId="10" r:id="R90157911225e477d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Digital" sheetId="11" r:id="R3ded539a9a67441d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Sostenib" sheetId="12" r:id="R2173d26ce4c14472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 IPE II" sheetId="13" r:id="Ra44c5eefacd44005"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Reparto" sheetId="14" r:id="Ra3e514278be14a1a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Itinerarios" sheetId="15" r:id="R5fcca5a5113849c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Auditoría" sheetId="16" r:id="Ra78e75c5f2ac4b3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Vertical mínimo" sheetId="17" r:id="R84d82f7b5baa4d22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Contrato firma" sheetId="18" r:id="R5db7995489384e3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Cambios" sheetId="19" r:id="R7015abb030474df6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00 Contrato" sheetId="1" r:id="Re808187cd6604fa6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 PI II" sheetId="2" r:id="R4f4ca0ee39164a7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 AD" sheetId="3" r:id="R2d79308cd72d4590"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 PMDM" sheetId="4" r:id="Rba3659c4b9e74a69"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 Hitos" sheetId="5" r:id="R2b1e9819021a4321"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="99 Guía" sheetId="6" r:id="R6aa065da43884f71"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 DI" sheetId="7" r:id="Ra35f1e510b92477a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 PSP" sheetId="8" r:id="R72fff220981444db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 SGE" sheetId="9" r:id="R8de2fd98c9934b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08 Nube" sheetId="10" r:id="R0574a93e778d45b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09 Digital" sheetId="11" r:id="Rea01c728c79c4e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10 Sostenib" sheetId="12" r:id="R9e86f924997d4ee9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11 IPE II" sheetId="13" r:id="Rcd4403c33442418e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12 Reparto" sheetId="14" r:id="R369dc4ef1a6c4320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13 Itinerarios" sheetId="15" r:id="R9147a80aaca745c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14 Auditoría" sheetId="16" r:id="Rc1c79a2e03f141cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="15 Vertical mínimo" sheetId="17" r:id="Ra060a5ee3f404aff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="16 Contrato firma" sheetId="18" r:id="R8f7775db70284d8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="17 Cambios" sheetId="19" r:id="R9fa8e70fca6046fe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1435,7 +1435,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rdf6a9ec96b64477d"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Raaaebba1dddb44cf"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -2573,7 +2573,7 @@
     <x:mergeCell ref="I26:K26"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R741b06e0106e4537"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432f74502e444e15"/>
 </x:worksheet>
 </file>
 
@@ -4819,7 +4819,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L42">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6572,7 +6572,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L27">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -8223,7 +8223,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L24">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -10012,7 +10012,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L28">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -14797,12 +14797,12 @@
       <x:formula1>"NO CONTRATADA,BACKLOG,PLANIFICADA,EN DESARROLLO,EN REVISIÓN,ACEPTADA,BLOQUEADA,RECUPERACIÓN"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L48">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc633ae8bb5ab451b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4873b7eafbbb452f"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -18115,12 +18115,12 @@
       <x:formula1>"NO CONTRATADA,BACKLOG,PLANIFICADA,EN DESARROLLO,EN REVISIÓN,ACEPTADA,BLOQUEADA,RECUPERACIÓN"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L67">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R46c964db5d3b4741"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfc8500f182aa4888"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -20411,12 +20411,12 @@
       <x:formula1>"NO CONTRATADA,BACKLOG,PLANIFICADA,EN DESARROLLO,EN REVISIÓN,ACEPTADA,BLOQUEADA,RECUPERACIÓN"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L49">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5edeb86b8e68447b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb17e97d29a014f02"/>
   </x:tableParts>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -23462,7 +23462,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L45">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -25623,7 +25623,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L39">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -27648,7 +27648,7 @@
       <x:formula1>"H0,H1,H2,H3,H4,H5"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="L15:L35">
-      <x:formula1>'00 Contrato'!$B$7:$B$9</x:formula1>
+      <x:formula1>'16 Contrato firma'!$B$7:$B$10</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>